<commit_message>
Rework optional item layout in wooden door quotation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GwKJzi7gcLve2q11GYhard
</commit_message>
<xml_diff>
--- a/quotes/Quotation_for_OPBM2-KW003D-01_Wooden_Door_for_APT.xlsx
+++ b/quotes/Quotation_for_OPBM2-KW003D-01_Wooden_Door_for_APT.xlsx
@@ -11,7 +11,7 @@
     <sheet name="QUOTATION" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">QUOTATION!$A$1:$G$27</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">QUOTATION!$A$1:$G$26</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -94,19 +94,20 @@
     <t xml:space="preserve">LOT</t>
   </si>
   <si>
-    <t xml:space="preserve">SUB TOTAL ($)</t>
+    <t xml:space="preserve">2*</t>
   </si>
   <si>
-    <t xml:space="preserve">OPTIONAL ITEM</t>
+    <t xml:space="preserve">Transport &amp; Installation
+(OPTIONAL)</t>
   </si>
   <si>
-    <t xml:space="preserve">Transport &amp; Installation</t>
+    <t xml:space="preserve">Delivery of doors to site and complete installation - at client's option</t>
   </si>
   <si>
-    <t xml:space="preserve">Delivery of doors to site and complete installation</t>
+    <t xml:space="preserve">TOTAL - SUPPLY ONLY ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">GRAND TOTAL ($) (incl. optional item)</t>
+    <t xml:space="preserve">TOTAL - SUPPLY + TRANSPORT &amp; INSTALLATION* ($)</t>
   </si>
   <si>
     <t xml:space="preserve">NOTES </t>
@@ -133,7 +134,7 @@
     <t xml:space="preserve">DELIVERY TERMS</t>
   </si>
   <si>
-    <t xml:space="preserve">Type-A: DDP Site; Type-B: Ex-Works Lagos (transport &amp; installation optional)</t>
+    <t xml:space="preserve">Type-A: DDP Site; Type-B: Ex-Works Lagos (*item 2 is optional, shaded)</t>
   </si>
   <si>
     <t xml:space="preserve">PAYMENT:</t>
@@ -827,6 +828,14 @@
       <charset val="1"/>
     </font>
     <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="14"/>
       <color theme="1"/>
@@ -851,16 +860,8 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
-    <font>
-      <i val="true"/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -871,6 +872,12 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.7999"/>
         <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -7207,7 +7214,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7324,27 +7331,55 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="89" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="86" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="89" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="240" fontId="89" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="241" fontId="89" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="241" fontId="89" fillId="3" borderId="1" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="90" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="241" fontId="89" fillId="0" borderId="8" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="241" fontId="90" fillId="0" borderId="8" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="90" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="90" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="241" fontId="90" fillId="3" borderId="8" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="91" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="17" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="91" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="92" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7352,15 +7387,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="86" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="86" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="92" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="89" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="92" fillId="4" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="89" fillId="5" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9377,7 +9412,7 @@
       <rgbColor rgb="FF00B0F0"/>
       <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFEDEDED"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFF2CC"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -9409,13 +9444,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>65880</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>794880</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>69840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -9429,7 +9464,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6464880" y="7009560"/>
+          <a:off x="6464880" y="6714360"/>
           <a:ext cx="794880" cy="3960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9446,13 +9481,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1776240</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>793800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>285480</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>1215000</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
@@ -9462,9 +9497,9 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3345840" y="7737480"/>
+          <a:off x="3345840" y="7442280"/>
           <a:ext cx="1194120" cy="421200"/>
-          <a:chOff x="3345840" y="7737480"/>
+          <a:chOff x="3345840" y="7442280"/>
           <a:chExt cx="1194120" cy="421200"/>
         </a:xfrm>
       </xdr:grpSpPr>
@@ -9479,7 +9514,7 @@
         </xdr:blipFill>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="3345840" y="7737480"/>
+            <a:off x="3345840" y="7442280"/>
             <a:ext cx="1194120" cy="421200"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
@@ -9840,330 +9875,329 @@
       </c>
       <c r="H12" s="24"/>
     </row>
-    <row r="13" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="29"/>
-      <c r="G13" s="30" t="n">
+      <c r="B13" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="32" t="n">
+        <v>5883</v>
+      </c>
+      <c r="G13" s="33" t="n">
+        <f aca="false">E13*F13</f>
+        <v>5883</v>
+      </c>
+      <c r="H13" s="24"/>
+    </row>
+    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="35" t="n">
         <f aca="false">G12</f>
         <v>98473.65</v>
       </c>
-      <c r="H13" s="24"/>
-    </row>
-    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="31"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
       <c r="H14" s="24"/>
     </row>
-    <row r="15" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
-        <v>2</v>
+    <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="36" t="s">
+        <v>27</v>
       </c>
-      <c r="B15" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>5883</v>
-      </c>
-      <c r="G15" s="28" t="n">
-        <f aca="false">E15*F15</f>
-        <v>5883</v>
+      <c r="B15" s="36"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="37" t="n">
+        <f aca="false">G12+G13</f>
+        <v>104356.65</v>
       </c>
       <c r="H15" s="24"/>
     </row>
-    <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29" t="s">
-        <v>27</v>
+    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="38"/>
+    </row>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="40" t="s">
+        <v>28</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="30" t="n">
-        <f aca="false">G13+G15</f>
-        <v>104356.65</v>
-      </c>
-      <c r="H16" s="24"/>
-    </row>
-    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="32"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
-        <v>28</v>
+      <c r="A18" s="41" t="s">
+        <v>29</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
+      <c r="B18" s="41"/>
+      <c r="C18" s="42" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="42"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="42"/>
+      <c r="G18" s="42"/>
       <c r="H18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34" t="s">
-        <v>29</v>
+      <c r="A19" s="41" t="s">
+        <v>31</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="35" t="s">
-        <v>30</v>
+      <c r="B19" s="41"/>
+      <c r="C19" s="42" t="s">
+        <v>32</v>
       </c>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
       <c r="H19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>31</v>
+      <c r="A20" s="41" t="s">
+        <v>33</v>
       </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="35" t="s">
-        <v>32</v>
+      <c r="B20" s="41"/>
+      <c r="C20" s="42" t="s">
+        <v>34</v>
       </c>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
       <c r="H20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="s">
-        <v>33</v>
+      <c r="A21" s="41" t="s">
+        <v>35</v>
       </c>
-      <c r="B21" s="34"/>
-      <c r="C21" s="35" t="s">
-        <v>34</v>
+      <c r="B21" s="41"/>
+      <c r="C21" s="42" t="s">
+        <v>36</v>
       </c>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
       <c r="H21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>35</v>
+      <c r="A22" s="41" t="s">
+        <v>37</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="35" t="s">
-        <v>36</v>
+      <c r="B22" s="41"/>
+      <c r="C22" s="42" t="s">
+        <v>38</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
       <c r="H22" s="24"/>
     </row>
-    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="34"/>
-      <c r="C23" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H23" s="24"/>
     </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="2.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H24" s="24"/>
     </row>
-    <row r="25" customFormat="false" ht="2.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="102.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="43"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
       <c r="H25" s="24"/>
     </row>
-    <row r="26" customFormat="false" ht="102.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="36" t="s">
-        <v>39</v>
+    <row r="26" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C26" s="24" t="s">
+        <v>40</v>
       </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="37"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="38"/>
-      <c r="G26" s="38"/>
       <c r="H26" s="24"/>
     </row>
-    <row r="27" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="H27" s="24"/>
+    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="38"/>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="38"/>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="32"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="32"/>
+      <c r="A28" s="38"/>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="38"/>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="32"/>
-      <c r="B29" s="32"/>
-      <c r="C29" s="32"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="32"/>
+      <c r="A29" s="38"/>
+      <c r="B29" s="38"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="38"/>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="32"/>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
+      <c r="A31" s="38"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="32"/>
-      <c r="B32" s="32"/>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
+      <c r="A32" s="38"/>
+      <c r="B32" s="38"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="32"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
+      <c r="A33" s="38"/>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="32"/>
+      <c r="A34" s="38"/>
+      <c r="B34" s="38"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="32"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
+      <c r="A35" s="38"/>
+      <c r="B35" s="38"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="32"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
+      <c r="A36" s="38"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="32"/>
+      <c r="A37" s="38"/>
+      <c r="B37" s="38"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="32"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="32"/>
+      <c r="A38" s="38"/>
+      <c r="B38" s="38"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="32"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-      <c r="F39" s="32"/>
-      <c r="G39" s="32"/>
-      <c r="H39" s="32"/>
+      <c r="A39" s="38"/>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="32"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-      <c r="H40" s="32"/>
+      <c r="A40" s="38"/>
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="19">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E1:G2"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="E7:F8"/>
     <mergeCell ref="G7:G8"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:G18"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C19:G19"/>
     <mergeCell ref="A20:B20"/>
@@ -10172,9 +10206,7 @@
     <mergeCell ref="C21:G21"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.472916666666667" right="0.290277777777778" top="1.44722222222222" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Restore Chrisbeth letterhead header images and footer in wooden door quotation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GwKJzi7gcLve2q11GYhard
</commit_message>
<xml_diff>
--- a/quotes/Quotation_for_OPBM2-KW003D-01_Wooden_Door_for_APT.xlsx
+++ b/quotes/Quotation_for_OPBM2-KW003D-01_Wooden_Door_for_APT.xlsx
@@ -10209,12 +10209,14 @@
     <mergeCell ref="A25:B25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.472916666666667" right="0.290277777777778" top="1.44722222222222" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.472916666666667" right="0.290277777777778" top="1.6" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="85" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter>&amp;LCHRISBETH QUOTATION&amp;C&amp;"Times New Roman,Bold"&amp;9 &amp;K00b0f0_x005F_x000a_&amp;R&amp;P</oddFooter>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;G&amp;R&amp;G</oddHeader>
+    <oddFooter>&amp;LCHRISBETH QUOTATION&amp;C&amp;"Times New Roman,Bold"&amp;9&amp;K00B0F0
+&amp;R&amp;P</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
+  <legacyDrawingHF r:id="rIdHF1"/>
 </worksheet>
 </file>
</xml_diff>